<commit_message>
Actualización automática 2026-09-18 13:30:21
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1587,10 +1587,10 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>-104.09</v>
+        <v>728.6</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>-81.23999999999999</v>
+        <v>2355.88</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -1614,10 +1614,10 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>0</v>
+        <v>2624.47</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>2504.1</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1845,7 +1845,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0</v>
+        <v>2203.11</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0</v>
@@ -2298,57 +2298,57 @@
     <row r="31">
       <c r="C31" s="3" t="inlineStr">
         <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>1 de 29</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
         <is>
           <t>0 de 29</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>2 de 29</t>
+          <t>3 de 29</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>2 de 29</t>
+          <t>3 de 29</t>
         </is>
       </c>
       <c r="N31" s="3" t="inlineStr">
@@ -2863,7 +2863,7 @@
         <v>10009.97</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>-185.33</v>
+        <v>8213.049999999999</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>0</v>
@@ -2971,7 +2971,7 @@
         <v>5615.24</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0</v>
+        <v>2209.88</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>0</v>
@@ -3204,7 +3204,7 @@
         <v>40471.33</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>4030.39</v>
+        <v>14638.65</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-09-21 08:30:19
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GONZALEZ CARDENAS ERNESTO PAOLO</t>
+          <t>GRANIMUNDO S.A.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GRANIMUNDO S.A.</t>
+          <t>LINO TUMBACO VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>LINO TUMBACO VICENTE JAVIER</t>
+          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
+          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1494,10 +1494,10 @@
         <v>0</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>0</v>
+        <v>423.26</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0</v>
+        <v>332.08</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -1523,14 +1523,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
+          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0</v>
+        <v>728.6</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0</v>
+        <v>2355.88</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
@@ -1554,10 +1554,10 @@
         <v>0</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>423.26</v>
+        <v>2624.47</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>332.08</v>
+        <v>2504.1</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -1583,14 +1583,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
+          <t>PAREDES ORTIZ MARIA INES</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>728.6</v>
+        <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>2355.88</v>
+        <v>0</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -1614,10 +1614,10 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>2624.47</v>
+        <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>2504.1</v>
+        <v>0</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PAREDES ORTIZ MARIA INES</t>
+          <t>RENOVA&amp;DISEÑA S.A.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1674,10 +1674,10 @@
         <v>0</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>0</v>
+        <v>457.23</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0</v>
+        <v>2908.35</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RENOVA&amp;DISEÑA S.A.</t>
+          <t>REYES AGUILERA JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1734,10 +1734,10 @@
         <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>457.23</v>
+        <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>2908.35</v>
+        <v>0</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>REYES AGUILERA JESSICA ELIZABETH</t>
+          <t>ROCA REYNA PAUL DAVID</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1785,7 +1785,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0</v>
+        <v>2203.11</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0</v>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ROCA REYNA PAUL DAVID</t>
+          <t>SANCHEZ SABANDO LUIS JAVIER</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1845,7 +1845,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>2203.11</v>
+        <v>0</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0</v>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SANCHEZ SABANDO LUIS JAVIER</t>
+          <t>SUMBA GARCIA MARCOS ANTONIO</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SUMBA GARCIA MARCOS ANTONIO</t>
+          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
+          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
+          <t>VERA ARCE MARIA ISABEL</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>VERA ARCE MARIA ISABEL</t>
+          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
+          <t>ZAMBRANO REYNA JOSE ALEJANDRO</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2236,144 +2236,84 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>MEZA PEÑA CARLOS ROBERTO</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>ZAMBRANO REYNA JOSE ALEJANDRO</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>1 de 29</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>1 de 29</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>1 de 29</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="L31" s="3" t="inlineStr">
-        <is>
-          <t>3 de 29</t>
-        </is>
-      </c>
-      <c r="M31" s="3" t="inlineStr">
-        <is>
-          <t>3 de 29</t>
-        </is>
-      </c>
-      <c r="N31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="O31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="P31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="Q31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
-        </is>
-      </c>
-      <c r="R31" s="3" t="inlineStr">
-        <is>
-          <t>0 de 29</t>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>1 de 28</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>1 de 28</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>1 de 28</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>3 de 28</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>3 de 28</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="inlineStr">
+        <is>
+          <t>0 de 28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-10-07 14:30:15
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1677,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0</v>
+        <v>45.49</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="M30" s="3" t="inlineStr">
         <is>
-          <t>0 de 28</t>
+          <t>1 de 28</t>
         </is>
       </c>
       <c r="N30" s="3" t="inlineStr">
@@ -2857,7 +2857,7 @@
         <v>3780.23</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0</v>
+        <v>45.49</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>0</v>
@@ -3144,7 +3144,7 @@
         <v>24236.5</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>571.54</v>
+        <v>617.03</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-16 08:30:18
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -683,7 +683,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ARBIZACONSTRUC S.A.</t>
+          <t>ARBOLEDA ZAMBRANO ROBERTO ANTONIO</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -743,7 +743,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ARBOLEDA ZAMBRANO ROBERTO ANTONIO</t>
+          <t>ARELLANO CEDEÑO DANNY MARCELO</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -803,7 +803,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ARELLANO CEDEÑO DANNY MARCELO</t>
+          <t>ARMIJOS BARCIA FRACISCO ANTONIO</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -863,7 +863,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ARMIJOS BARCIA FRACISCO ANTONIO</t>
+          <t>BAESCORP S.A.S.</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -923,7 +923,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BAESCORP S.A.S.</t>
+          <t>CEDEÑO ALAVA SANDRA ELIZABETH</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CEDEÑO ALAVA SANDRA ELIZABETH</t>
+          <t>CHANGKUON AYON JOSE CRISTOBAL</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CHANGKUON AYON JOSE CRISTOBAL</t>
+          <t>DELGADO COPPIANO JORGE RODOLFO</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DELGADO COPPIANO JORGE RODOLFO</t>
+          <t>FERRETERIA UNIDA ZAMBRANO FERRUZAM CIA. LTDA.</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FERRETERIA UNIDA ZAMBRANO FERRUZAM CIA. LTDA.</t>
+          <t>FREILE FERRIN FRECIA NOEMI LOURDE</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FREILE FERRIN FRECIA NOEMI LOURDE</t>
+          <t>GRANIMUNDO S.A.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GRANIMUNDO S.A.</t>
+          <t>LINO TUMBACO VICENTE JAVIER</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>LINO TUMBACO VICENTE JAVIER</t>
+          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MANABITA DE REPUESTOS MANARECO C LTDA</t>
+          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MATERIALES PARA DECORACION DECORCASA CIA. LTDA.</t>
+          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MOREIRA MOREIRA PATRICIO IGNACIO</t>
+          <t>PAREDES ORTIZ MARIA INES</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PAREDES ORTIZ MARIA INES</t>
+          <t>RENOVA&amp;DISEÑA S.A.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1617,7 +1617,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>45.49</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>RENOVA&amp;DISEÑA S.A.</t>
+          <t>REYES AGUILERA JESSICA ELIZABETH</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1677,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>45.49</v>
+        <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>REYES AGUILERA JESSICA ELIZABETH</t>
+          <t>ROCA REYNA PAUL DAVID</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1734,7 +1734,7 @@
         <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>0</v>
+        <v>571.54</v>
       </c>
       <c r="M21" s="2" t="n">
         <v>0</v>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ROCA REYNA PAUL DAVID</t>
+          <t>SANCHEZ SABANDO LUIS JAVIER</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1794,7 +1794,7 @@
         <v>0</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>571.54</v>
+        <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
         <v>0</v>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SANCHEZ SABANDO LUIS JAVIER</t>
+          <t>SUMBA GARCIA MARCOS ANTONIO</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SUMBA GARCIA MARCOS ANTONIO</t>
+          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1943,7 +1943,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>TUTIVEN PAREDES MARCIA PIEDAD</t>
+          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>VACA CANCHINGRE FATIMA YAQUELINE</t>
+          <t>VERA ARCE MARIA ISABEL</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>VERA ARCE MARIA ISABEL</t>
+          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ZAMBRANO FERNANDEZ JOSE LUIS</t>
+          <t>ZAMBRANO REYNA JOSE ALEJANDRO</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2176,144 +2176,84 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>MEZA PEÑA CARLOS ROBERTO</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>ZAMBRANO REYNA JOSE ALEJANDRO</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="L30" s="3" t="inlineStr">
-        <is>
-          <t>1 de 28</t>
-        </is>
-      </c>
-      <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>1 de 28</t>
-        </is>
-      </c>
-      <c r="N30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="O30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="P30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="Q30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
-        </is>
-      </c>
-      <c r="R30" s="3" t="inlineStr">
-        <is>
-          <t>0 de 28</t>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>1 de 27</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>1 de 27</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
+        </is>
+      </c>
+      <c r="R29" s="3" t="inlineStr">
+        <is>
+          <t>0 de 27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-10-19 17:30:17
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -2797,7 +2797,7 @@
         <v>3780.23</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>45.49</v>
+        <v>71.27</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
         <v>24236.5</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>617.03</v>
+        <v>642.8099999999999</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-28 08:30:16
</commit_message>
<xml_diff>
--- a/data/MEZA PEÑA CARLOS ROBERTO.xlsx
+++ b/data/MEZA PEÑA CARLOS ROBERTO.xlsx
@@ -1734,13 +1734,13 @@
         <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>5058.09</v>
+        <v>5380.97</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0</v>
+        <v>21.8</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0</v>
+        <v>914.4</v>
       </c>
       <c r="O21" s="2" t="n">
         <v>0</v>
@@ -2228,12 +2228,12 @@
       </c>
       <c r="M29" s="3" t="inlineStr">
         <is>
+          <t>2 de 27</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
           <t>1 de 27</t>
-        </is>
-      </c>
-      <c r="N29" s="3" t="inlineStr">
-        <is>
-          <t>0 de 27</t>
         </is>
       </c>
       <c r="O29" s="3" t="inlineStr">
@@ -2851,7 +2851,7 @@
         <v>2894.56</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>5058.09</v>
+        <v>6317.17</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
         <v>24236.5</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>13884.48</v>
+        <v>15143.56</v>
       </c>
       <c r="G30" s="4" t="n">
         <v>0</v>

</xml_diff>